<commit_message>
Hoàn thiện 3.1 bệnh án, chẩn đoán
</commit_message>
<xml_diff>
--- a/clinic/docs/master-plan/Master Plan.xlsx
+++ b/clinic/docs/master-plan/Master Plan.xlsx
@@ -1756,12 +1756,12 @@
         <v>19</v>
       </c>
       <c r="E10" s="15"/>
-      <c r="F10" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="20">
-        <v>1</v>
-      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>Tạm hoãn</t>
+        </is>
+      </c>
+      <c r="G10" s="20"/>
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
@@ -1840,12 +1840,12 @@
         <v>19</v>
       </c>
       <c r="E11" s="6"/>
-      <c r="F11" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="20">
-        <v>1</v>
-      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Tạm hoãn</t>
+        </is>
+      </c>
+      <c r="G11" s="20"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
@@ -2258,11 +2258,13 @@
         <v>19</v>
       </c>
       <c r="E16" s="23"/>
-      <c r="F16" s="19" t="s">
-        <v>20</v>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>Tạm hoãn</t>
+        </is>
       </c>
       <c r="G16" s="20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
@@ -4417,7 +4419,7 @@
       <formula1>"10%,20%,30%,40%,50%,60%,70%,80%,90%,100%"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F4:F17 F19:F27 F29:F30" xr:uid="{00000000-0002-0000-0000-000001000000}">
-      <formula1>"Đang thực hiện,Đã hoàn thành"</formula1>
+      <formula1>"Đang thực hiện,Đã hoàn thành,Tạm hoãn"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>